<commit_message>
DONE training the model
</commit_message>
<xml_diff>
--- a/backend/files/forecastData/user_3/forecast_summary_20251114_205438.xlsx
+++ b/backend/files/forecastData/user_3/forecast_summary_20251114_205438.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\kgs-sales-forecasting\backend\files\forecastData\user_3\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1345996C-FDC1-4081-818F-2119B728C0C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{303AAB40-7CE1-4DDC-9F78-FD578981EF14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="7d_forecast" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -94,7 +94,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -400,7 +400,8 @@
   <dimension ref="A1:C8"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="3" width="17.6640625" customWidth="1"/>
+    <col min="1" max="1" width="22" customWidth="1"/>
+    <col min="2" max="3" width="17.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
@@ -852,7 +853,7 @@
   <dimension ref="A1:C91"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="20.21875" customWidth="1"/>
+    <col min="1" max="1" width="23" customWidth="1"/>
     <col min="2" max="3" width="16.21875" customWidth="1"/>
   </cols>
   <sheetData>

</xml_diff>